<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.002-06 Le manteau jaune de Raphaël
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.002-06.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.002-06.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le nez rose du chat</t>
+          <t>Le manteau jaune de Raphaël</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine au cacao, puis classe</t>
+          <t>maison sous la pluie, gouttière, cacao, bottes, classe</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Raphaël, papa, maman, maîtresse</t>
+          <t>Raphaël, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Raphaël veut raconter le chat du radiateur. Le mot est déjà là. Il lève la main, il attend, puis il parle.</t>
+          <t>Une vapeur de cacao danse près de la vitre. Sur le bouton, un éclat de manteau brille. Raphaël veut parler maintenant. Il coupe papa : les mots se perdent. Il enfile trop vite : le bouton manque. À l'école, sa phrase se cogne à la classe. Il refuse de foncer, attend le silence, raconte le chat. Merci vécu. Sur le bouton, l'éclat de manteau tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La casserole chante tout bas. Une buée monte sur la vitre. Le cacao sent le chocolat chaud. Une mousse brune fait un petit chapeau. Raphaël, souffle un peu. C'est encore trop chaud. Ça sent trop bon. Le chat s'est mis sur le radiateur. Le chat est gris, tout rond. Son nez est rose, tout petit. Il ronronne, comme un moteur doux. Il est tout chaud. Oui. Il aime le radiateur. Tu veux le raconter à l'école ? Oui. Le nez est rose. Le crayon gris, dans la poche. Raphaël glisse le crayon. Le bois est lisse, un peu froid. On met le manteau. Le jaune, celui-là. Un bouton. Puis l'autre. Le tissu est froid. On ouvre. L'air sent la terre mouillée. Une goutte tombe du rebord. Tic. Tu restes près de moi. D'accord, maman. Les bottes font un bruit mou. L'école a une porte en bois. Le couloir sent la laine mouillée. Le crochet est à ta hauteur. Raphaël accroche le manteau. Il goutte encore un peu. Au revoir, Raphaël. Au revoir, papa. On revient tout à l'heure. Au revoir, maman. En ce moment, Raphaël s'assoit. Le tapis bleu est un peu frais. Il pose les mains sur ses genoux. Le crayon gris reste dans la poche. La maîtresse ouvre un grand livre. Une image d'animaux apparaît. Bonjour. Bonjour. Qui a vu un animal, ce matin ? Raphaël a une idée. Le chat du radiateur. Le nez rose, tout petit. Le mot est déjà là. Il ouvre un peu la bouche. La maîtresse tourne encore une page. Le papier fait un petit bruit.</t>
+          <t>Une vapeur de cacao danse près de la vitre. La vitre est tiède, un peu floue. Le manteau jaune attend sur la chaise. Sur le bouton, un éclat de manteau brille. Il est blanc, papa. C'est le fil, sous la lumière. Papa glisse les bottes rouges près de la porte. Tes lacets, Raphaël ? Maman noue un lacet, puis l'autre. Ça sent le cacao, chaud. Le chat gris dort sur le radiateur. Son nez est rose, minuscule. Il ronronne, papa. Tu l'entends, Raphaël ? Oui. Je le dis à l'école ! Tu l'entends, la gouttière ? Elle chante. Elle boit la pluie. Papa, le bouton brille, maintenant ! Papa parle à maman, près des bottes. Les bottes sont mouillées, pour dehors. Les mots de Raphaël se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Raphaël ? Le bouton. Il brille. En ce moment, Raphaël pose la main sur le manteau. Le tissu est rêche, un peu froid. Je le mets, maintenant ! Il enfile le manteau trop vite. Le bouton manque. Le capuchon penche sur l'œil. Oh. L'éclat de manteau tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. On boutonne ensemble ? Oui, papa. Ils avancent jusqu'à la porte. Tu dis bonjour, à l'école ? Oui, maman. Au revoir, maman. Au revoir, Raphaël. Dehors, la gouttière chante sur le toit. La pluie dessine des fils gris. Les gouttes tapent sur le capuchon. Ça chante sur ma tête. Oui. C'est la pluie. L'air sent la terre. Les bottes font un bruit mou. L'école a une porte en bois. Le couloir sent la laine mouillée. Une petite flaque brille sous la botte. Le crochet est à ta hauteur. Raphaël accroche le manteau. On revient te chercher. Au revoir, papa. Le tapis de la classe est bleu. Il est un peu frais sous les genoux. Les cubes en bois sentent la forêt. Le doudou lapin reste dans le sac. Raphaël s'assoit sur le tapis. Il pose les mains sur ses genoux. La maîtresse parle près des chaises. Bonjour, maîtresse. Une image d'animaux attend sur le livre. Raphaël a une idée. Le chat de la maison est gris. Son nez est rose. Je le dis, maintenant ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne comprend. Raphaël referme la bouche. Il serre les mains sur ses genoux.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La casserole chante tout bas. Une buée monte sur la vitre. Le cacao sent le chocolat chaud. Une mousse brune fait un petit chapeau. Raphaël, souffle un peu. C'est encore trop chaud. Ça sent trop bon. Le chat s'est mis sur le radiateur. Le chat est gris, tout rond. Son nez est rose, tout petit. Il ronronne, comme un moteur doux. Il est tout chaud. Oui. Il aime le radiateur. Tu veux le raconter à l'école ? Oui. Le nez est rose. Le crayon gris, dans la poche. Raphaël glisse le crayon. Le bois est lisse, un peu froid. On met le manteau. Le jaune, celui-là. Un bouton. Puis l'autre. Le tissu est froid. On ouvre. L'air sent la terre mouillée. Une goutte tombe du rebord. Tic. Tu restes près de moi. D'accord, maman. Les bottes font un bruit mou. L'école a une porte en bois. Le couloir sent la laine mouillée. Le crochet est à ta hauteur. Raphaël accroche le manteau. Il goutte encore un peu. Au revoir, Raphaël. Au revoir, papa. On revient tout à l'heure. Au revoir, maman. En ce moment, Raphaël s'assoit. Le tapis bleu est un peu frais. Il pose les mains sur ses genoux. Le crayon gris reste dans la poche. La maîtresse ouvre un grand livre. Une image d'animaux apparaît. Bonjour. Bonjour. Qui a vu un animal, ce matin ? Raphaël a une idée. Le chat du radiateur. Le nez rose, tout petit. Le mot est déjà là. Il ouvre un peu la bouche. La maîtresse tourne encore une page. Le papier fait un petit bruit.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une vapeur de cacao danse près de la vitre. La vitre est tiède, un peu floue. Le manteau jaune attend sur la chaise. Sur le bouton, un &lt;emphasis level="moderate"&gt;éclat de manteau&lt;/emphasis&gt; brille. Il est blanc, papa. C'est le fil, sous la lumière. Papa glisse les bottes rouges près de la porte. Tes lacets, Raphaël ? Maman noue un lacet, puis l'autre. Ça sent le cacao, chaud. Le chat gris dort sur le radiateur. Son nez est rose, minuscule. Il ronronne, papa. Tu l'entends, Raphaël ? Oui. Je le dis à l'école ! Tu l'entends, la gouttière ? Elle chante. Elle boit la pluie. Papa, le bouton brille, maintenant ! Papa parle à maman, près des bottes. Les bottes sont mouillées, pour dehors. Les mots de Raphaël se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Raphaël ? Le bouton. Il brille. En ce moment, Raphaël pose la main sur le manteau. Le tissu est rêche, un peu froid. Je le mets, maintenant ! Il enfile le manteau trop vite. Le bouton manque. Le capuchon penche sur l'œil. Oh. L'éclat de manteau tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. On boutonne ensemble ? Oui, papa. Ils avancent jusqu'à la porte. Tu dis bonjour, à l'école ? Oui, maman. Au revoir, maman. Au revoir, Raphaël. Dehors, la gouttière chante sur le toit. La pluie dessine des fils gris. Les gouttes tapent sur le capuchon. Ça chante sur ma tête. Oui. C'est la pluie. L'air sent la terre. Les bottes font un bruit mou. L'école a une porte en bois. Le couloir sent la laine mouillée. Une petite flaque brille sous la botte. Le crochet est à ta hauteur. Raphaël accroche le manteau. On revient te chercher. Au revoir, papa. Le tapis de la classe est bleu. Il est un peu frais sous les genoux. Les cubes en bois sentent la forêt. Le doudou lapin reste dans le sac. Raphaël s'assoit sur le tapis. Il pose les mains sur ses genoux. La maîtresse parle près des chaises. Bonjour, maîtresse. Une image d'animaux attend sur le livre. Raphaël a une idée. Le chat de la maison est gris. Son nez est rose. Je le dis, maintenant ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne comprend. Raphaël referme la bouche. Il serre les mains sur ses genoux.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Élie arrive en classe avec maman. Maman dit au revoir. Élie s'assoit sur le tapis. La maîtresse pose une question. Élie a une idée. Il lève la main. Il faut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Un camarade parle d'abord. Élie attend encore. Puis la maîtresse dit : Élie, c'est ton tour. Élie parle. Il dit : le chat est gris. La maîtresse sourit. Le soir, maman demande. Élie dit : j'ai levé la main. J'ai su attendre. Puis j'ai parlé. Maman dit : merci Élie. Attendre, puis parler.&lt;/slow&gt; [pause]</t>
+          <t>Une vapeur de cacao danse près de la vitre. La vitre est tiède, un peu floue. Le manteau jaune attend sur la chaise. Sur le bouton, un &lt;emphasis&gt;éclat de manteau&lt;/emphasis&gt; brille. Il est blanc, papa. C'est le fil, sous la lumière. Papa glisse les bottes rouges près de la porte. Tes lacets, Raphaël ? Maman noue un lacet, puis l'autre. Ça sent le cacao, chaud. Le chat gris dort sur le radiateur. Son nez est rose, minuscule. Il ronronne, papa. Tu l'entends, Raphaël ? Oui. Je le dis à l'école ! Tu l'entends, la gouttière ? Elle chante. Elle boit la pluie. Papa, le bouton brille, maintenant ! Papa parle à maman, près des bottes. Les bottes sont mouillées, pour dehors. Les mots de Raphaël se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Raphaël ? Le bouton. Il brille. En ce moment, Raphaël pose la main sur le manteau. Le tissu est rêche, un peu froid. Je le mets, maintenant ! Il enfile le manteau trop vite. Le bouton manque. Le capuchon penche sur l'œil. Oh. L'éclat de manteau tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. On boutonne ensemble ? Oui, papa. Ils avancent jusqu'à la porte. Tu dis bonjour, à l'école ? Oui, maman. Au revoir, maman. Au revoir, Raphaël. Dehors, la gouttière chante sur le toit. La pluie dessine des fils gris. Les gouttes tapent sur le capuchon. Ça chante sur ma tête. Oui. C'est la pluie. L'air sent la terre. Les bottes font un bruit mou. L'école a une porte en bois. Le couloir sent la laine mouillée. Une petite flaque brille sous la botte. Le crochet est à ta hauteur. Raphaël accroche le manteau. On revient te chercher. Au revoir, papa. Le tapis de la classe est bleu. Il est un peu frais sous les genoux. Les cubes en bois sentent la forêt. Le doudou lapin reste dans le sac. Raphaël s'assoit sur le tapis. Il pose les mains sur ses genoux. La maîtresse parle près des chaises. Bonjour, maîtresse. Une image d'animaux attend sur le livre. Raphaël a une idée. Le chat de la maison est gris. Son nez est rose. Je le dis, maintenant ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne comprend. Raphaël referme la bouche. Il serre les mains sur ses genoux. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de manteau</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,73 +1324,100 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_parler_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La casserole chante tout bas.
-narrateur|Une buée monte sur la vitre.
-narrateur|Le cacao sent le chocolat chaud.
-narrateur|Une mousse brune fait un petit chapeau.
-papa|Raphaël, souffle un peu.
-papa|C'est encore trop chaud.
-enfant-m|Ça sent trop bon.
-maman|Le chat s'est mis sur le radiateur.
-narrateur|Le chat est gris, tout rond.
-narrateur|Son nez est rose, tout petit.
-narrateur|Il ronronne, comme un moteur doux.
-enfant-m|Il est tout chaud.
-maman|Oui.
-maman|Il aime le radiateur.
-papa|Tu veux le raconter à l'école ?
+          <t>narrateur|Une vapeur de cacao danse près de la vitre.
+narrateur|La vitre est tiède, un peu floue.
+narrateur|Le manteau jaune attend sur la chaise.
+narrateur|Sur le bouton, un éclat de manteau brille.
+enfant-m|Il est blanc, papa.
+papa|C'est le fil, sous la lumière.
+narrateur|Papa glisse les bottes rouges près de la porte.
+maman|Tes lacets, Raphaël ?
+narrateur|Maman noue un lacet, puis l'autre.
+narrateur|Ça sent le cacao, chaud.
+narrateur|Le chat gris dort sur le radiateur.
+narrateur|Son nez est rose, minuscule.
+enfant-m|Il ronronne, papa.
+papa|Tu l'entends, Raphaël ?
 enfant-m|Oui.
-enfant-m|Le nez est rose.
-maman|Le crayon gris, dans la poche.
-narrateur|Raphaël glisse le crayon.
-narrateur|Le bois est lisse, un peu froid.
-papa|On met le manteau.
-papa|Le jaune, celui-là.
-maman|Un bouton.
-maman|Puis l'autre.
-enfant-m|Le tissu est froid.
-papa|On ouvre.
-narrateur|L'air sent la terre mouillée.
-narrateur|Une goutte tombe du rebord.
-narrateur|Tic.
-maman|Tu restes près de moi.
-enfant-m|D'accord, maman.
+enfant-m|Je le dis à l'école !
+maman|Tu l'entends, la gouttière ?
+enfant-m|Elle chante.
+papa|Elle boit la pluie.
+enfant-m|Papa, le bouton brille, maintenant !
+narrateur|Papa parle à maman, près des bottes.
+papa|Les bottes sont mouillées, pour dehors.
+narrateur|Les mots de Raphaël se cognent aux leurs.
+narrateur|Personne ne tourne la tête.
+papa|Tu disais quelque chose, Raphaël ?
+enfant-m|Le bouton.
+enfant-m|Il brille.
+narrateur|En ce moment, Raphaël pose la main sur le manteau.
+narrateur|Le tissu est rêche, un peu froid.
+enfant-m|Je le mets, maintenant !
+narrateur|Il enfile le manteau trop vite.
+narrateur|Le bouton manque.
+narrateur|Le capuchon penche sur l'œil.
+enfant-m|Oh.
+narrateur|L'éclat de manteau tremble, puis tient.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Ça ne veut pas, maman.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|On boutonne ensemble ?
+enfant-m|Oui, papa.
+narrateur|Ils avancent jusqu'à la porte.
+maman|Tu dis bonjour, à l'école ?
+enfant-m|Oui, maman.
+enfant-m|Au revoir, maman.
+maman|Au revoir, Raphaël.
+narrateur|Dehors, la gouttière chante sur le toit.
+narrateur|La pluie dessine des fils gris.
+narrateur|Les gouttes tapent sur le capuchon.
+enfant-m|Ça chante sur ma tête.
+papa|Oui.
+papa|C'est la pluie.
+narrateur|L'air sent la terre.
 narrateur|Les bottes font un bruit mou.
 narrateur|L'école a une porte en bois.
 narrateur|Le couloir sent la laine mouillée.
+narrateur|Une petite flaque brille sous la botte.
 maman|Le crochet est à ta hauteur.
 narrateur|Raphaël accroche le manteau.
-maman|Il goutte encore un peu.
-papa|Au revoir, Raphaël.
+papa|On revient te chercher.
 enfant-m|Au revoir, papa.
-maman|On revient tout à l'heure.
-enfant-m|Au revoir, maman.
-narrateur|En ce moment, Raphaël s'assoit.
-narrateur|Le tapis bleu est un peu frais.
+narrateur|Le tapis de la classe est bleu.
+narrateur|Il est un peu frais sous les genoux.
+narrateur|Les cubes en bois sentent la forêt.
+narrateur|Le doudou lapin reste dans le sac.
+narrateur|Raphaël s'assoit sur le tapis.
 narrateur|Il pose les mains sur ses genoux.
-narrateur|Le crayon gris reste dans la poche.
-narrateur|La maîtresse ouvre un grand livre.
-narrateur|Une image d'animaux apparaît.
-maitresse|Bonjour.
-enfant-m|Bonjour.
-maitresse|Qui a vu un animal, ce matin ?
+narrateur|La maîtresse parle près des chaises.
+enfant-m|Bonjour, maîtresse.
+narrateur|Une image d'animaux attend sur le livre.
 narrateur|Raphaël a une idée.
-narrateur|Le chat du radiateur.
-narrateur|Le nez rose, tout petit.
-narrateur|Le mot est déjà là.
-narrateur|Il ouvre un peu la bouche.
-narrateur|La maîtresse tourne encore une page.
-narrateur|Le papier fait un petit bruit.</t>
+narrateur|Le chat de la maison est gris.
+narrateur|Son nez est rose.
+enfant-m|Je le dis, maintenant !
+narrateur|Il ouvre la bouche trop vite.
+narrateur|Ses mots se cognent à la classe.
+narrateur|Personne ne comprend.
+narrateur|Raphaël referme la bouche.
+narrateur|Il serre les mains sur ses genoux.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>casserole,pluie,pas</t>
+          <t>pluie,gouttiere,pas</t>
         </is>
       </c>
     </row>
@@ -1422,12 +1449,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël veut parler. Que fait-il d'abord ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Raphaël veut &lt;emphasis level="moderate"&gt;parler&lt;/emphasis&gt;. Que fait-il d'abord ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Élie veut parler. Que fait-il d'abord ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Raphaël veut &lt;emphasis&gt;parler&lt;/emphasis&gt;. Que fait-il d'abord ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1490,7 +1517,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1498,10 +1525,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1516,34 +1543,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>parler</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1552,13 +1583,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1568,7 +1599,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_parle_quand_le_silence_arrive; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1601,17 +1632,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël lève la main. Sa main reste en l'air. Il attend. La maîtresse parle encore du livre. Raphaël regarde une goutte sur la vitre. Sa main ne descend pas. Le crayon reste dans la poche. Raphaël, c'est toi. Tu peux parler. Le chat est gris. Il était sur le radiateur. Son nez est rose. Raphaël montre le crayon gris. Un nez rose, tout petit. Oui. Il ronronnait. Merci, Raphaël. Raphaël repose le crayon. Le bois est encore lisse.</t>
+          <t>Raphaël ouvre la bouche trop vite. Le chat est gris ! Une voix d'enfant parle près du tapis. On entend un lapin blanc. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Les mains se posent à plat. Une main monte, sans crier. Sa main reste en l'air. Il regarde la pluie sur la vitre. Le tapis bleu est frais sous les genoux. Un cube de bois roule, puis s'arrête. Le lapin blanc finit sa phrase. Un silence arrive près du tapis. Derrière la porte, le manteau jaune attend. Sur le bouton, l'éclat de manteau brille. Je peux dire quelque chose ? La maîtresse tourne la tête, près du livre. Le chat est gris. Il a un nez rose. Il aime le radiateur. La classe écoute jusqu'au bout. Raphaël montre le bout de son doigt. Minuscule, comme ça. Le ventre de Raphaël se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël lève la main. Sa main reste en l'air. Il attend. La maîtresse parle encore du livre. Raphaël regarde une goutte sur la vitre. Sa main ne descend pas. Le crayon reste dans la poche. Raphaël, c'est toi. Tu peux parler. Le chat est gris. Il était sur le radiateur. Son nez est rose. Raphaël montre le crayon gris. Un nez rose, tout petit. Oui. Il ronronnait. Merci, Raphaël. Raphaël repose le crayon. Le bois est encore lisse.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël ouvre la bouche trop vite. Le chat est gris ! Une voix d'enfant parle près du tapis. On entend un lapin blanc. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Les mains se posent à plat. Une main monte, sans crier. Sa main reste en l'air. Il regarde la pluie sur la vitre. Le tapis bleu est frais sous les genoux. Un cube de bois roule, puis s'arrête. Le lapin blanc finit sa phrase. Un &lt;emphasis level="moderate"&gt;silence&lt;/emphasis&gt; arrive près du tapis. Derrière la porte, le manteau jaune attend. Sur le bouton, l'éclat de manteau brille. Je peux dire quelque chose ? La maîtresse tourne la tête, près du livre. Le chat est gris. Il a un nez rose. Il aime le radiateur. La classe écoute jusqu'au bout. Raphaël montre le bout de son doigt. Minuscule, comme ça. Le ventre de Raphaël se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Élie a levé la main. Il a attendu. &lt;emphasis&gt;puis&lt;/emphasis&gt; il a parlé. C'était son tour.&lt;/slow&gt; [pause]</t>
+          <t>Raphaël ouvre la bouche trop vite. Le chat est gris ! Une voix d'enfant parle près du tapis. On entend un lapin blanc. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Les mains se posent à plat. Une main monte, sans crier. Sa main reste en l'air. Il regarde la pluie sur la vitre. Le tapis bleu est frais sous les genoux. Un cube de bois roule, puis s'arrête. Le lapin blanc finit sa phrase. Un &lt;emphasis&gt;silence&lt;/emphasis&gt; arrive près du tapis. Derrière la porte, le manteau jaune attend. Sur le bouton, l'éclat de manteau brille. Je peux dire quelque chose ? La maîtresse tourne la tête, près du livre. Le chat est gris. Il a un nez rose. Il aime le radiateur. La classe écoute jusqu'au bout. Raphaël montre le bout de son doigt. Minuscule, comme ça. Le ventre de Raphaël se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1658,18 +1689,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1692,30 +1723,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>puis</t>
+          <t>silence</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1724,10 +1755,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1736,34 +1767,43 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_attend_puis_on_l_entend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël lève la main.
+          <t>narrateur|Raphaël ouvre la bouche trop vite.
+enfant-m|Le chat est gris !
+narrateur|Une voix d'enfant parle près du tapis.
+narrateur|On entend un lapin blanc.
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Raphaël refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Les mains se posent à plat.
+narrateur|Une main monte, sans crier.
 narrateur|Sa main reste en l'air.
-narrateur|Il attend.
-narrateur|La maîtresse parle encore du livre.
-narrateur|Raphaël regarde une goutte sur la vitre.
-narrateur|Sa main ne descend pas.
-narrateur|Le crayon reste dans la poche.
-maitresse|Raphaël, c'est toi.
-maitresse|Tu peux parler.
+narrateur|Il regarde la pluie sur la vitre.
+narrateur|Le tapis bleu est frais sous les genoux.
+narrateur|Un cube de bois roule, puis s'arrête.
+narrateur|Le lapin blanc finit sa phrase.
+narrateur|Un silence arrive près du tapis.
+narrateur|Derrière la porte, le manteau jaune attend.
+narrateur|Sur le bouton, l'éclat de manteau brille.
+enfant-m|Je peux dire quelque chose ?
+narrateur|La maîtresse tourne la tête, près du livre.
 enfant-m|Le chat est gris.
-enfant-m|Il était sur le radiateur.
-enfant-m|Son nez est rose.
-narrateur|Raphaël montre le crayon gris.
-maitresse|Un nez rose, tout petit.
-enfant-m|Oui.
-enfant-m|Il ronronnait.
-maitresse|Merci, Raphaël.
-narrateur|Raphaël repose le crayon.
-narrateur|Le bois est encore lisse.</t>
+enfant-m|Il a un nez rose.
+enfant-m|Il aime le radiateur.
+narrateur|La classe écoute jusqu'au bout.
+narrateur|Raphaël montre le bout de son doigt.
+enfant-m|Minuscule, comme ça.
+narrateur|Le ventre de Raphaël se desserre.</t>
         </is>
       </c>
     </row>
@@ -1790,17 +1830,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, une petite cloche sonne. Raphaël range son cartable. Le manteau jaune est presque sec. La porte s'ouvre. Tu as passé un bon moment ? J'ai parlé du chat. Son nez est rose. Il était sur le radiateur ? Oui, papa. On rentre. La pluie est plus douce. Les bottes font un petit bruit. La maison sent encore le cacao. Le chat est déjà sur le radiateur. Il est encore là. Oui. Tout rond. Tu bois une gorgée, d'abord. Raphaël souffle sur le cacao. Puis il raconte le nez rose. Je t'écoute.</t>
+          <t>Plus tard, une petite cloche sonne. Raphaël range son cartable. Le manteau jaune est presque sec. La porte s'ouvre. Tu as passé un bon moment ? Le chat ! Le nez rose ! Les bottes, Raphaël ? Les deux voix se mélangent. Oh. Il saisit le manteau trop vite. Le capuchon penche. Oh. Les mots se perdent dans le couloir. Raphaël s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Le manteau revient contre sa poitrine. Il écoute la gouttière, un instant. Je peux te dire quelque chose ? Oui, nous t'écoutons. J'ai parlé du chat. Après le lapin blanc. Merci, Raphaël. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le capuchon, tu le vois ? Oui, papa. Le bois du crochet tient le jaune. Raphaël enfile le manteau, sans tirer. Les bottes, maintenant ? Je les mets. Les bottes font un petit bruit. On rentre. La pluie tape plus doucement.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, une petite cloche sonne. Raphaël range son cartable. Le manteau jaune est presque sec. La porte s'ouvre. Tu as passé un bon moment ? J'ai parlé du chat. Son nez est rose. Il était sur le radiateur ? Oui, papa. On rentre. La pluie est plus douce. Les bottes font un petit bruit. La maison sent encore le cacao. Le chat est déjà sur le radiateur. Il est encore là. Oui. Tout rond. Tu bois une gorgée, d'abord. Raphaël souffle sur le cacao. Puis il raconte le nez rose. Je t'écoute.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus tard, une petite cloche sonne. Raphaël range son cartable. Le &lt;emphasis level="moderate"&gt;manteau&lt;/emphasis&gt; jaune est presque sec. La porte s'ouvre. Tu as passé un bon moment ? Le chat ! Le nez rose ! Les bottes, Raphaël ? Les deux voix se mélangent. Oh. Il saisit le manteau trop vite. Le capuchon penche. Oh. Les mots se perdent dans le couloir. Raphaël s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Le manteau revient contre sa poitrine. Il écoute la gouttière, un instant. Je peux te dire quelque chose ? Oui, nous t'écoutons. J'ai parlé du chat. Après le lapin blanc. Merci, Raphaël. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le capuchon, tu le vois ? Oui, papa. Le bois du crochet tient le jaune. Raphaël enfile le manteau, sans tirer. Les bottes, maintenant ? Je les mets. Les bottes font un petit bruit. On rentre. La pluie tape plus doucement.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Élie range son cartable. Maman l'attend à la porte.&lt;/slow&gt; [pause]</t>
+          <t>Plus tard, une petite cloche sonne. Raphaël range son cartable. Le &lt;emphasis&gt;manteau&lt;/emphasis&gt; jaune est presque sec. La porte s'ouvre. Tu as passé un bon moment ? Le chat ! Le nez rose ! Les bottes, Raphaël ? Les deux voix se mélangent. Oh. Il saisit le manteau trop vite. Le capuchon penche. Oh. Les mots se perdent dans le couloir. Raphaël s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Le manteau revient contre sa poitrine. Il écoute la gouttière, un instant. Je peux te dire quelque chose ? Oui, nous t'écoutons. J'ai parlé du chat. Après le lapin blanc. Merci, Raphaël. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le capuchon, tu le vois ? Oui, papa. Le bois du crochet tient le jaune. Raphaël enfile le manteau, sans tirer. Les bottes, maintenant ? Je les mets. Les bottes font un petit bruit. On rentre. La pluie tape plus doucement. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1847,18 +1887,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1879,28 +1919,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>manteau</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1909,10 +1953,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1921,9 +1965,13 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sur_le_manteau; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
           <t>narrateur|Plus tard, une petite cloche sonne.
@@ -1931,22 +1979,37 @@
 narrateur|Le manteau jaune est presque sec.
 narrateur|La porte s'ouvre.
 maman|Tu as passé un bon moment ?
+enfant-m|Le chat !
+enfant-m|Le nez rose !
+papa|Les bottes, Raphaël ?
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Il saisit le manteau trop vite.
+narrateur|Le capuchon penche.
+enfant-m|Oh.
+narrateur|Les mots se perdent dans le couloir.
+narrateur|Raphaël s'arrête.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Il refuse de foncer.
+narrateur|Le manteau revient contre sa poitrine.
+narrateur|Il écoute la gouttière, un instant.
+enfant-m|Je peux te dire quelque chose ?
+maman|Oui, nous t'écoutons.
 enfant-m|J'ai parlé du chat.
-enfant-m|Son nez est rose.
-papa|Il était sur le radiateur ?
+enfant-m|Après le lapin blanc.
+papa|Merci, Raphaël.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu as soif ?
+enfant-m|Un peu, maman.
+papa|Le capuchon, tu le vois ?
 enfant-m|Oui, papa.
-maman|On rentre.
-narrateur|La pluie est plus douce.
+narrateur|Le bois du crochet tient le jaune.
+narrateur|Raphaël enfile le manteau, sans tirer.
+maman|Les bottes, maintenant ?
+enfant-m|Je les mets.
 narrateur|Les bottes font un petit bruit.
-narrateur|La maison sent encore le cacao.
-narrateur|Le chat est déjà sur le radiateur.
-enfant-m|Il est encore là.
-papa|Oui.
-papa|Tout rond.
-maman|Tu bois une gorgée, d'abord.
-narrateur|Raphaël souffle sur le cacao.
-narrateur|Puis il raconte le nez rose.
-maman|Je t'écoute.</t>
+papa|On rentre.
+narrateur|La pluie tape plus doucement.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1978,17 +2041,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le chat ronronne sur le radiateur. Le crayon gris repose près de la tasse. Bonne soirée, mon grand. Le nez était rose. Oui.</t>
+          <t>Le manteau jaune sèche sur le crochet. L'air sent le cacao, plus loin. Il a fait tout le chemin. Toi aussi. La pluie est plus douce, près de la vitre. Tu souffles ? Oui, maman. Raphaël souffle. Le ventre est large, à sa place. On est bien, ici. Les bottes sèchent près de la porte. Je les verrai. Le chat gris dort sur le radiateur. Son nez est rose. Oui. Le doudou lapin est dans le lit. L'éclat de manteau tient sur le bouton.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le chat ronronne sur le radiateur. Le crayon gris repose près de la tasse. Bonne soirée, mon grand. Le nez était rose. Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le manteau jaune sèche sur le crochet. L'air sent le cacao, plus loin. Il a fait tout le chemin. Toi aussi. La pluie est plus douce, près de la vitre. Tu souffles ? Oui, maman. Raphaël souffle. Le ventre est large, à sa place. On est bien, ici. Les bottes sèchent près de la porte. Je les verrai. Le chat gris dort sur le radiateur. Son nez est rose. Oui. Le doudou lapin est dans le lit. L'&lt;emphasis level="moderate"&gt;éclat de manteau&lt;/emphasis&gt; tient sur le bouton.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le manteau jaune sèche sur le crochet. L'air sent le cacao, plus loin. Il a fait tout le chemin. Toi aussi. La pluie est plus douce, près de la vitre. Tu souffles ? Oui, maman. Raphaël souffle. Le ventre est large, à sa place. On est bien, ici. Les bottes sèchent près de la porte. Je les verrai. Le chat gris dort sur le radiateur. Son nez est rose. Oui. Le doudou lapin est dans le lit. L'&lt;emphasis&gt;éclat de manteau&lt;/emphasis&gt; tient sur le bouton.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2035,7 +2098,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2043,10 +2106,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2055,12 +2118,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2069,17 +2132,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de manteau</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2088,11 +2155,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2101,28 +2168,44 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bouton; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le chat ronronne sur le radiateur.
-narrateur|Le crayon gris repose près de la tasse.
-maman|Bonne soirée, mon grand.
-papa|Le nez était rose.
-enfant-m|Oui.</t>
+          <t>narrateur|Le manteau jaune sèche sur le crochet.
+narrateur|L'air sent le cacao, plus loin.
+enfant-m|Il a fait tout le chemin.
+papa|Toi aussi.
+narrateur|La pluie est plus douce, près de la vitre.
+maman|Tu souffles ?
+enfant-m|Oui, maman.
+narrateur|Raphaël souffle.
+narrateur|Le ventre est large, à sa place.
+maman|On est bien, ici.
+papa|Les bottes sèchent près de la porte.
+enfant-m|Je les verrai.
+narrateur|Le chat gris dort sur le radiateur.
+enfant-m|Son nez est rose.
+papa|Oui.
+narrateur|Le doudou lapin est dans le lit.
+narrateur|L'éclat de manteau tient sur le bouton.</t>
         </is>
       </c>
     </row>
@@ -2143,7 +2226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2228,6 +2311,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>